<commit_message>
Anúncio por referência, PDF do calendário e painel no celular
- Anúncios: criativo pode ser "Referência" ou "Arte final" (ads.creative_stage),
  no cadastro, na seleção em massa e na planilha; portal mostra a etiqueta e
  lê por portal_ad_list()
- Portal: botão "Baixar PDF" gera no navegador o mês em grade e a lista completa
- Painel no celular: menu com ícone acima do nome, nome do usuário inteiro,
  títulos da lista em até 3 linhas, barra de ações em massa sem cortes
- Testes e capturas do painel no celular (ux-admin-shots)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BfwzxzGkpZoptqEjU2AfmT
</commit_message>
<xml_diff>
--- a/site/admin/modelo-importacao-anuncios.xlsx
+++ b/site/admin/modelo-importacao-anuncios.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -455,9 +455,10 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
     <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -518,22 +519,27 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Tipo do criativo</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Observação para o cliente</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Observações internas</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Enviar para aprovação</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Meta Ads,Google Ads,TikTok Ads"</formula1>
     </dataValidation>
@@ -543,7 +549,10 @@
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Reconhecimento da marca,Tráfego para o site,Engajamento,Cadastros (leads),Vendas,Mensagens,Outro"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Referência,Arte final"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -557,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -840,7 +849,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Observação para o cliente</t>
+          <t>Tipo do criativo</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -850,19 +859,19 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Aparece para o cliente nos detalhes do anúncio</t>
+          <t>Referência = o cliente aprova a ideia/inspiração (a arte final vai depois, como nova versão). Arte final = pronta para veicular. Vazio: com link do criativo, conta como Referência</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Confira o preço antes de aprovar</t>
+          <t>Referência</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Observações internas</t>
+          <t>Observação para o cliente</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -872,56 +881,78 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Só a equipe vê</t>
+          <t>Aparece para o cliente nos detalhes do anúncio</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Verba de R$ 500</t>
+          <t>Confira o preço antes de aprovar</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>Observações internas</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Só a equipe vê</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Verba de R$ 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>Enviar para aprovação</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Sim = já vai para o cliente aprovar (precisa ter link do criativo). Não ou vazio = entra como rascunho</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Sim</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-    </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="4" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Dica</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>A primeira linha precisa ter os títulos das colunas. A ordem das colunas não importa e colunas a mais são ignoradas. Antes de gravar, o painel mostra uma prévia com o que está pronto e o que precisa de correção.</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Anúncio por referência sem arquivo: só o escopo e a ideia escritos
- Banco: ad_transition aceita enviar uma referência sem arquivo/link quando
  o escopo está preenchido (sem_escopo); arte final continua exigindo criativo
- Painel: campo "Escopo, ideia e referências", avisos e envio em massa com a
  mesma regra (adCanSend)
- Portal: card "Ideia e escopo", texto com quebras de linha e sem prévia vazia
- Planilha: coluna "Escopo, ideia e referências"; marcado para enviar sem link
  entra como referência
- Revoga a função antiga portal_ads()
- Testes do envio sem arquivo (painel, banco emulado e portal)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BfwzxzGkpZoptqEjU2AfmT
</commit_message>
<xml_diff>
--- a/site/admin/modelo-importacao-anuncios.xlsx
+++ b/site/admin/modelo-importacao-anuncios.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Contexto da campanha</t>
+          <t>Escopo, ideia e referências</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -695,7 +695,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Contexto da campanha</t>
+          <t>Escopo, ideia e referências</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -705,12 +705,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Para quem é, período, oferta (até 2.000 caracteres)</t>
+          <t>Para quem é, período, oferta, o que será criado, a ideia e as referências em texto (até 2.000 caracteres). O cliente lê. Com isto preenchido, uma Referência pode ir para aprovação sem link</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Clientes que já compraram. Julho.</t>
+          <t>Clientes que já compraram, julho. Foto do balcão com luz da manhã, tons quentes, estilo dos posts da @exemplo.</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Referência = o cliente aprova a ideia/inspiração (a arte final vai depois, como nova versão). Arte final = pronta para veicular. Vazio: com link do criativo, conta como Referência</t>
+          <t>Referência = o cliente aprova a ideia/inspiração (a arte final vai depois, como nova versão). Arte final = pronta para veicular. Vazio: com link do criativo, ou marcado para enviar, conta como Referência</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Sim = já vai para o cliente aprovar (precisa ter link do criativo). Não ou vazio = entra como rascunho</t>
+          <t>Sim = já vai para o cliente aprovar (arte final precisa de link do criativo; referência pode ir só com o escopo escrito). Não ou vazio = entra como rascunho</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">

</xml_diff>